<commit_message>
Replace the fisher groupoid experiment with geodesic_align so the branch snapshot matches the current mapping workflow.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/sample/sample_template.xlsx
+++ b/docs/sample/sample_template.xlsx
@@ -5,22 +5,36 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\my_github\excel-template-viz\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\my_github\excel-template-viz\docs\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F6AA3DD-D8F5-4354-87DD-0BC3CD98DA05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2402210-795A-4485-AC07-B633D63D295E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2730" windowWidth="28800" windowHeight="15345" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34920" yWindow="3270" windowWidth="21075" windowHeight="15345" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Input_sheet" sheetId="1" r:id="rId1"/>
     <sheet name="Print_sheet" sheetId="2" r:id="rId2"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId3"/>
+  </externalReferences>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">Print_sheet!$A$1:$B$8</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">Print_sheet!$B$1:$C$9</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -32,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="21">
   <si>
     <t>ID#</t>
   </si>
@@ -52,9 +66,6 @@
     <t>Sign</t>
   </si>
   <si>
-    <t>Clark Kent</t>
-  </si>
-  <si>
     <t>recreate himself without changing his dob on records</t>
   </si>
   <si>
@@ -83,6 +94,26 @@
   </si>
   <si>
     <t>Effective_Date</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Last name</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>First name</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Kent</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Clark</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>name combination</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -133,11 +164,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="176" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -153,6 +187,33 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="sheet1"/>
+      <sheetName val="sheet2"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="4">
+          <cell r="B4" t="str">
+            <v>Kent</v>
+          </cell>
+          <cell r="C4" t="str">
+            <v>Clark</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -265,84 +326,113 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="5.42578125" customWidth="1"/>
-    <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="4" width="72.7109375" customWidth="1"/>
-    <col min="5" max="5" width="26.85546875" customWidth="1"/>
-    <col min="6" max="6" width="10.42578125" customWidth="1"/>
-    <col min="7" max="7" width="5.140625" customWidth="1"/>
+    <col min="1" max="4" width="5.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="52.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.85546875" customWidth="1"/>
+    <col min="9" max="9" width="10.42578125" customWidth="1"/>
+    <col min="10" max="10" width="5.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>8129</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="1" t="str">
+        <f>[1]sheet1!$C$4 &amp; [1]sheet1!$B$4</f>
+        <v>ClarkKent</v>
+      </c>
+      <c r="E2" s="1" t="str">
+        <f>IF(D2="",C2&amp;" "&amp;B2,D2)</f>
+        <v>ClarkKent</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="I2" s="2">
+        <v>46053</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="2">
-        <v>46053</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>250</v>
       </c>
       <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="1" t="str">
+        <f>[1]sheet1!$C$7 &amp; [1]sheet1!$B$7</f>
+        <v/>
+      </c>
+      <c r="E3" s="1" t="str">
+        <f>IF(D3="",C3&amp;" "&amp;B3,D3)</f>
+        <v xml:space="preserve"> 狗蛋</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="G3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="H3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="2">
+      <c r="I3" s="2">
         <v>46053</v>
       </c>
-      <c r="G3" s="1" t="s">
-        <v>10</v>
+      <c r="J3" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -358,77 +448,108 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="1" max="1" width="13.7109375" customWidth="1"/>
     <col min="2" max="2" width="31.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="str">
+        <f>"The ticket  for " &amp; TEXT(C1,"str")</f>
+        <v>The ticket  for ClarkKent</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+      <c r="C1" s="1" t="str">
+        <f>Input_sheet!E2</f>
+        <v>ClarkKent</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="4"/>
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2">
-        <v>28550</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+      <c r="C2" s="2" t="str">
+        <f>Input_sheet!G2</f>
+        <v>1978/02/29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="4"/>
+      <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="2">
-        <v>46023</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
+      <c r="C3" s="1" t="str">
+        <f>Input_sheet!H2</f>
+        <v>10 Years of Community Service</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="4"/>
+      <c r="B4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="2">
+        <f>Input_sheet!I2</f>
+        <v>46053</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B5" s="1"/>
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="str">
+        <f>"The ticket  for " &amp; TEXT(C6,"str")</f>
+        <v>The ticket  for  狗蛋</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
+      <c r="C6" t="str">
+        <f>Input_sheet!E3</f>
+        <v xml:space="preserve"> 狗蛋</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="4"/>
+      <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="2">
-        <v>47484</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
+      <c r="C7" s="2" t="str">
+        <f>Input_sheet!G3</f>
+        <v>2026/01/31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="4"/>
+      <c r="B8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C8" s="1" t="str">
+        <f>Input_sheet!H3</f>
+        <v>Brush teeth daily</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="4"/>
+      <c r="B9" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="2">
+      <c r="C9" s="2">
+        <f>Input_sheet!I3</f>
         <v>46053</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:A4"/>
+    <mergeCell ref="A6:A9"/>
+  </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -437,7 +558,7 @@
     <oddFooter>&amp;C&amp;"Times New Roman,标准"&amp;12页 &amp;P</oddFooter>
   </headerFooter>
   <rowBreaks count="1" manualBreakCount="1">
-    <brk id="4" max="1" man="1"/>
+    <brk id="5" min="1" max="2" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
</xml_diff>